<commit_message>
Update AkbariHo mapping, Launcher ports, and ManseokHo error logic
</commit_message>
<xml_diff>
--- a/낚시 오픈일.xlsx
+++ b/낚시 오픈일.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\gemini\fishing_bot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB8A1BD9-B1BD-4CEA-B589-B5696C1FA3D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0999AAB9-D530-4342-91D9-A9E2FB69B594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{148B82DD-3426-458A-916A-D3FE202A9A2C}"/>
+    <workbookView xWindow="1210" yWindow="0" windowWidth="13860" windowHeight="17280" xr2:uid="{148B82DD-3426-458A-916A-D3FE202A9A2C}"/>
   </bookViews>
   <sheets>
     <sheet name="작성자_DK" sheetId="1" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2233" uniqueCount="1067">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2245" uniqueCount="1079">
   <si>
     <t>선사</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -4133,6 +4133,54 @@
     <t>만석선단</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
+  <si>
+    <t>10일전</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1월 31일(토) 12시</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>만수피싱</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2월 01일(일) 06시</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>베스트피싱</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2월 01일(일) 07시</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>영진호</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>평택항</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2월 01일(일) 09시</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>오닉스호</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2월 01일(일) 11시</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>크루즈호</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -4142,7 +4190,7 @@
     <numFmt numFmtId="176" formatCode="&quot;₩&quot;#,##0"/>
     <numFmt numFmtId="177" formatCode="mm&quot;월&quot;\ dd&quot;일&quot;"/>
   </numFmts>
-  <fonts count="34">
+  <fonts count="33">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4395,17 +4443,8 @@
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <u/>
-      <sz val="12"/>
-      <color rgb="FFFF0000"/>
-      <name val="맑은 고딕"/>
-      <family val="2"/>
-      <charset val="129"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="17">
+  <fills count="18">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -4499,6 +4538,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -4660,7 +4705,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="101">
+  <cellXfs count="102">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -4901,15 +4946,6 @@
     <xf numFmtId="0" fontId="31" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -4962,6 +4998,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -5290,7 +5338,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A39E8B7-AF51-4CA2-AF7F-525187CC5D56}">
-  <dimension ref="B2:AA53"/>
+  <dimension ref="B2:AA58"/>
   <sheetFormatPr defaultRowHeight="17"/>
   <cols>
     <col min="1" max="1" width="3.4140625" customWidth="1"/>
@@ -5340,7 +5388,7 @@
       <c r="G2" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="H2" s="92" t="s">
+      <c r="H2" s="89" t="s">
         <v>1034</v>
       </c>
       <c r="I2" s="1" t="s">
@@ -5414,7 +5462,7 @@
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="6"/>
-      <c r="H3" s="93" t="s">
+      <c r="H3" s="90" t="s">
         <v>78</v>
       </c>
       <c r="I3" s="2"/>
@@ -5425,7 +5473,7 @@
       <c r="L3" s="2">
         <v>1</v>
       </c>
-      <c r="M3" s="84" t="s">
+      <c r="M3" s="81" t="s">
         <v>32</v>
       </c>
       <c r="N3" s="20" t="s">
@@ -5482,7 +5530,7 @@
       <c r="G4" s="2" t="s">
         <v>764</v>
       </c>
-      <c r="H4" s="94"/>
+      <c r="H4" s="91"/>
       <c r="I4" s="6"/>
       <c r="J4" s="6" t="s">
         <v>1036</v>
@@ -5546,7 +5594,7 @@
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="6"/>
-      <c r="H5" s="94"/>
+      <c r="H5" s="91"/>
       <c r="I5" s="6"/>
       <c r="J5" s="6" t="s">
         <v>1036</v>
@@ -5614,9 +5662,9 @@
         <v>65</v>
       </c>
       <c r="G6" s="6"/>
-      <c r="H6" s="94"/>
+      <c r="H6" s="91"/>
       <c r="I6" s="6"/>
-      <c r="J6" s="99" t="s">
+      <c r="J6" s="96" t="s">
         <v>1037</v>
       </c>
       <c r="K6" s="51"/>
@@ -5644,7 +5692,7 @@
       <c r="S6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="T6" s="84" t="s">
+      <c r="T6" s="81" t="s">
         <v>54</v>
       </c>
       <c r="U6" s="6" t="s">
@@ -5670,9 +5718,9 @@
       <c r="E7" s="6"/>
       <c r="F7" s="6"/>
       <c r="G7" s="6"/>
-      <c r="H7" s="94"/>
+      <c r="H7" s="91"/>
       <c r="I7" s="6"/>
-      <c r="J7" s="99" t="s">
+      <c r="J7" s="96" t="s">
         <v>1037</v>
       </c>
       <c r="K7" s="51"/>
@@ -5734,7 +5782,7 @@
       <c r="E8" s="6"/>
       <c r="F8" s="6"/>
       <c r="G8" s="6"/>
-      <c r="H8" s="94"/>
+      <c r="H8" s="91"/>
       <c r="I8" s="6"/>
       <c r="J8" s="6" t="s">
         <v>1036</v>
@@ -5800,7 +5848,7 @@
       <c r="G9" s="6" t="s">
         <v>439</v>
       </c>
-      <c r="H9" s="94"/>
+      <c r="H9" s="91"/>
       <c r="I9" s="6" t="s">
         <v>1018</v>
       </c>
@@ -5859,7 +5907,7 @@
       <c r="B10" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="C10" s="97" t="s">
+      <c r="C10" s="94" t="s">
         <v>103</v>
       </c>
       <c r="D10" s="14" t="s">
@@ -5872,8 +5920,8 @@
       <c r="G10" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="H10" s="94"/>
-      <c r="I10" s="96" t="s">
+      <c r="H10" s="91"/>
+      <c r="I10" s="93" t="s">
         <v>1015</v>
       </c>
       <c r="J10" s="6" t="s">
@@ -5934,7 +5982,7 @@
         <v>156</v>
       </c>
       <c r="G11" s="6"/>
-      <c r="H11" s="94" t="s">
+      <c r="H11" s="91" t="s">
         <v>78</v>
       </c>
       <c r="I11" s="6"/>
@@ -6010,9 +6058,9 @@
       <c r="G12" s="6" t="s">
         <v>437</v>
       </c>
-      <c r="H12" s="94"/>
+      <c r="H12" s="91"/>
       <c r="I12" s="6"/>
-      <c r="J12" s="99" t="s">
+      <c r="J12" s="96" t="s">
         <v>1037</v>
       </c>
       <c r="K12" s="51"/>
@@ -6065,7 +6113,7 @@
       <c r="B13" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="C13" s="97" t="s">
+      <c r="C13" s="94" t="s">
         <v>9</v>
       </c>
       <c r="D13" s="14" t="s">
@@ -6076,8 +6124,8 @@
         <v>152</v>
       </c>
       <c r="G13" s="6"/>
-      <c r="H13" s="94"/>
-      <c r="I13" s="96" t="s">
+      <c r="H13" s="91"/>
+      <c r="I13" s="93" t="s">
         <v>1018</v>
       </c>
       <c r="J13" s="6" t="s">
@@ -6146,7 +6194,7 @@
       <c r="G14" s="6" t="s">
         <v>438</v>
       </c>
-      <c r="H14" s="94"/>
+      <c r="H14" s="91"/>
       <c r="I14" s="6"/>
       <c r="J14" s="6" t="s">
         <v>1036</v>
@@ -6210,7 +6258,7 @@
       <c r="E15" s="6"/>
       <c r="F15" s="6"/>
       <c r="G15" s="6"/>
-      <c r="H15" s="94"/>
+      <c r="H15" s="91"/>
       <c r="I15" s="6"/>
       <c r="J15" s="6" t="s">
         <v>1036</v>
@@ -6252,9 +6300,9 @@
       <c r="G16" s="6" t="s">
         <v>437</v>
       </c>
-      <c r="H16" s="94"/>
+      <c r="H16" s="91"/>
       <c r="I16" s="6"/>
-      <c r="J16" s="99" t="s">
+      <c r="J16" s="96" t="s">
         <v>1037</v>
       </c>
       <c r="K16" s="51"/>
@@ -6276,9 +6324,7 @@
       <c r="Q16" s="30" t="s">
         <v>531</v>
       </c>
-      <c r="R16" s="4" t="s">
-        <v>91</v>
-      </c>
+      <c r="R16" s="4"/>
       <c r="S16" s="4" t="s">
         <v>105</v>
       </c>
@@ -6314,7 +6360,7 @@
         <v>449</v>
       </c>
       <c r="G17" s="6"/>
-      <c r="H17" s="94" t="s">
+      <c r="H17" s="91" t="s">
         <v>78</v>
       </c>
       <c r="I17" s="6"/>
@@ -6340,9 +6386,7 @@
       <c r="Q17" s="30" t="s">
         <v>532</v>
       </c>
-      <c r="R17" s="4" t="s">
-        <v>92</v>
-      </c>
+      <c r="R17" s="4"/>
       <c r="S17" s="4" t="s">
         <v>105</v>
       </c>
@@ -6376,9 +6420,9 @@
         <v>449</v>
       </c>
       <c r="G18" s="6"/>
-      <c r="H18" s="94"/>
+      <c r="H18" s="91"/>
       <c r="I18" s="6"/>
-      <c r="J18" s="99" t="s">
+      <c r="J18" s="96" t="s">
         <v>1037</v>
       </c>
       <c r="K18" s="51"/>
@@ -6400,9 +6444,7 @@
       <c r="Q18" s="30" t="s">
         <v>1021</v>
       </c>
-      <c r="R18" s="4" t="s">
-        <v>1011</v>
-      </c>
+      <c r="R18" s="4"/>
       <c r="S18" s="4" t="s">
         <v>105</v>
       </c>
@@ -6436,12 +6478,12 @@
       <c r="G19" s="57" t="s">
         <v>524</v>
       </c>
-      <c r="H19" s="95"/>
+      <c r="H19" s="92"/>
       <c r="I19" s="57"/>
       <c r="J19" s="6" t="s">
         <v>1036</v>
       </c>
-      <c r="K19" s="83"/>
+      <c r="K19" s="80"/>
       <c r="L19" s="6">
         <v>17</v>
       </c>
@@ -6506,7 +6548,7 @@
         <v>449</v>
       </c>
       <c r="G20" s="6"/>
-      <c r="H20" s="94"/>
+      <c r="H20" s="91"/>
       <c r="I20" s="6"/>
       <c r="J20" s="6" t="s">
         <v>1036</v>
@@ -6530,9 +6572,7 @@
       <c r="Q20" s="30" t="s">
         <v>533</v>
       </c>
-      <c r="R20" s="4" t="s">
-        <v>91</v>
-      </c>
+      <c r="R20" s="4"/>
       <c r="S20" s="4" t="s">
         <v>105</v>
       </c>
@@ -6566,7 +6606,7 @@
         <v>431</v>
       </c>
       <c r="G21" s="6"/>
-      <c r="H21" s="94"/>
+      <c r="H21" s="91"/>
       <c r="I21" s="6"/>
       <c r="J21" s="6" t="s">
         <v>1036</v>
@@ -6590,9 +6630,7 @@
       <c r="Q21" s="30" t="s">
         <v>534</v>
       </c>
-      <c r="R21" s="4" t="s">
-        <v>92</v>
-      </c>
+      <c r="R21" s="4"/>
       <c r="S21" s="4" t="s">
         <v>105</v>
       </c>
@@ -6626,7 +6664,7 @@
         <v>449</v>
       </c>
       <c r="G22" s="6"/>
-      <c r="H22" s="94" t="s">
+      <c r="H22" s="91" t="s">
         <v>58</v>
       </c>
       <c r="I22" s="6"/>
@@ -6652,9 +6690,7 @@
       <c r="Q22" s="30" t="s">
         <v>139</v>
       </c>
-      <c r="R22" s="4" t="s">
-        <v>91</v>
-      </c>
+      <c r="R22" s="4"/>
       <c r="S22" s="4" t="s">
         <v>105</v>
       </c>
@@ -6688,7 +6724,7 @@
       <c r="G23" s="2" t="s">
         <v>764</v>
       </c>
-      <c r="H23" s="94"/>
+      <c r="H23" s="91"/>
       <c r="I23" s="6"/>
       <c r="J23" s="6" t="s">
         <v>1036</v>
@@ -6712,9 +6748,7 @@
       <c r="Q23" s="30" t="s">
         <v>140</v>
       </c>
-      <c r="R23" s="4" t="s">
-        <v>92</v>
-      </c>
+      <c r="R23" s="4"/>
       <c r="S23" s="4" t="s">
         <v>105</v>
       </c>
@@ -6748,7 +6782,7 @@
         <v>65</v>
       </c>
       <c r="G24" s="6"/>
-      <c r="H24" s="94"/>
+      <c r="H24" s="91"/>
       <c r="I24" s="6"/>
       <c r="J24" s="6" t="s">
         <v>1036</v>
@@ -6772,9 +6806,7 @@
       <c r="Q24" s="30" t="s">
         <v>535</v>
       </c>
-      <c r="R24" s="4" t="s">
-        <v>91</v>
-      </c>
+      <c r="R24" s="4"/>
       <c r="S24" s="4" t="s">
         <v>105</v>
       </c>
@@ -6797,7 +6829,7 @@
       <c r="B25" s="14" t="s">
         <v>759</v>
       </c>
-      <c r="C25" s="97" t="s">
+      <c r="C25" s="14" t="s">
         <v>89</v>
       </c>
       <c r="D25" s="14" t="s">
@@ -6812,8 +6844,8 @@
       <c r="G25" s="6" t="s">
         <v>761</v>
       </c>
-      <c r="H25" s="94"/>
-      <c r="I25" s="96" t="s">
+      <c r="H25" s="91"/>
+      <c r="I25" s="101" t="s">
         <v>1017</v>
       </c>
       <c r="J25" s="6" t="s">
@@ -6838,9 +6870,7 @@
       <c r="Q25" s="30" t="s">
         <v>536</v>
       </c>
-      <c r="R25" s="4" t="s">
-        <v>92</v>
-      </c>
+      <c r="R25" s="4"/>
       <c r="S25" s="4" t="s">
         <v>105</v>
       </c>
@@ -6876,25 +6906,27 @@
       <c r="G26" s="6" t="s">
         <v>990</v>
       </c>
-      <c r="H26" s="94"/>
-      <c r="I26" s="6"/>
+      <c r="H26" s="91"/>
+      <c r="I26" s="6" t="s">
+        <v>1067</v>
+      </c>
       <c r="J26" s="6" t="s">
         <v>1036</v>
       </c>
       <c r="K26" s="51"/>
       <c r="L26" s="51"/>
       <c r="Q26" s="16"/>
-      <c r="R26" s="85"/>
+      <c r="R26" s="82"/>
       <c r="AA26" s="16"/>
     </row>
     <row r="27" spans="2:27">
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="14" t="s">
         <v>425</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="C27" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="D27" s="14" t="s">
         <v>6</v>
       </c>
       <c r="E27" s="6" t="s">
@@ -6904,7 +6936,7 @@
         <v>65</v>
       </c>
       <c r="G27" s="6"/>
-      <c r="H27" s="94"/>
+      <c r="H27" s="91"/>
       <c r="I27" s="6"/>
       <c r="J27" s="6" t="s">
         <v>1036</v>
@@ -6912,7 +6944,7 @@
       <c r="K27" s="51"/>
       <c r="L27" s="51"/>
       <c r="Q27" s="16"/>
-      <c r="R27" s="86"/>
+      <c r="R27" s="83"/>
       <c r="AA27" s="16"/>
     </row>
     <row r="28" spans="2:27">
@@ -6928,7 +6960,7 @@
       <c r="E28" s="6"/>
       <c r="F28" s="6"/>
       <c r="G28" s="6"/>
-      <c r="H28" s="94"/>
+      <c r="H28" s="91"/>
       <c r="I28" s="6"/>
       <c r="J28" s="6" t="s">
         <v>1036</v>
@@ -6936,7 +6968,7 @@
       <c r="K28" s="51"/>
       <c r="L28" s="51"/>
       <c r="Q28" s="16"/>
-      <c r="R28" s="86"/>
+      <c r="R28" s="83"/>
       <c r="W28" s="36">
         <f>SUM(W3:W27)</f>
         <v>1880000</v>
@@ -6956,7 +6988,7 @@
       <c r="E29" s="6"/>
       <c r="F29" s="6"/>
       <c r="G29" s="6"/>
-      <c r="H29" s="94"/>
+      <c r="H29" s="91"/>
       <c r="I29" s="6"/>
       <c r="J29" s="6" t="s">
         <v>1036</v>
@@ -6964,23 +6996,23 @@
       <c r="K29" s="51"/>
       <c r="L29" s="51"/>
       <c r="Q29" s="16"/>
-      <c r="R29" s="86"/>
+      <c r="R29" s="83"/>
       <c r="AA29" s="16"/>
     </row>
     <row r="30" spans="2:27">
       <c r="B30" s="4" t="s">
-        <v>1028</v>
+        <v>1068</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>1030</v>
+        <v>1069</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>1032</v>
+        <v>6</v>
       </c>
       <c r="E30" s="6"/>
       <c r="F30" s="6"/>
       <c r="G30" s="6"/>
-      <c r="H30" s="94"/>
+      <c r="H30" s="91"/>
       <c r="I30" s="6"/>
       <c r="J30" s="6" t="s">
         <v>1036</v>
@@ -6992,21 +7024,21 @@
     </row>
     <row r="31" spans="2:27" ht="17.5" thickBot="1">
       <c r="B31" s="4" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>523</v>
+        <v>1032</v>
       </c>
       <c r="E31" s="6"/>
       <c r="F31" s="6"/>
       <c r="G31" s="6"/>
-      <c r="H31" s="94"/>
+      <c r="H31" s="91"/>
       <c r="I31" s="6"/>
-      <c r="J31" s="99" t="s">
-        <v>1037</v>
+      <c r="J31" s="6" t="s">
+        <v>1036</v>
       </c>
       <c r="K31" s="51"/>
       <c r="M31" s="1" t="s">
@@ -7055,21 +7087,21 @@
     </row>
     <row r="32" spans="2:27" ht="17.5" thickTop="1">
       <c r="B32" s="4" t="s">
-        <v>991</v>
+        <v>1029</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>992</v>
+        <v>1031</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>6</v>
+        <v>523</v>
       </c>
       <c r="E32" s="6"/>
       <c r="F32" s="6"/>
       <c r="G32" s="6"/>
-      <c r="H32" s="94"/>
+      <c r="H32" s="91"/>
       <c r="I32" s="6"/>
-      <c r="J32" s="6" t="s">
-        <v>1036</v>
+      <c r="J32" s="96" t="s">
+        <v>1037</v>
       </c>
       <c r="K32" s="51"/>
       <c r="M32" s="20" t="s">
@@ -7114,21 +7146,21 @@
     </row>
     <row r="33" spans="2:27">
       <c r="B33" s="4" t="s">
-        <v>1038</v>
+        <v>991</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>1039</v>
+        <v>992</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>996</v>
+        <v>6</v>
       </c>
       <c r="E33" s="6"/>
       <c r="F33" s="6"/>
       <c r="G33" s="6"/>
-      <c r="H33" s="94"/>
+      <c r="H33" s="91"/>
       <c r="I33" s="6"/>
-      <c r="J33" s="99" t="s">
-        <v>1037</v>
+      <c r="J33" s="6" t="s">
+        <v>1036</v>
       </c>
       <c r="K33" s="51"/>
       <c r="M33" s="7" t="s">
@@ -7175,21 +7207,21 @@
     </row>
     <row r="34" spans="2:27">
       <c r="B34" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>84</v>
+        <v>1070</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>1071</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>8</v>
+        <v>1074</v>
       </c>
       <c r="E34" s="6"/>
       <c r="F34" s="6"/>
       <c r="G34" s="6"/>
-      <c r="H34" s="94"/>
+      <c r="H34" s="91"/>
       <c r="I34" s="6"/>
-      <c r="J34" s="99" t="s">
-        <v>1037</v>
+      <c r="J34" s="6" t="s">
+        <v>1036</v>
       </c>
       <c r="K34" s="51"/>
       <c r="M34" s="18" t="s">
@@ -7234,22 +7266,18 @@
     </row>
     <row r="35" spans="2:27">
       <c r="B35" s="4" t="s">
-        <v>85</v>
+        <v>1072</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>96</v>
+        <v>1073</v>
       </c>
       <c r="D35" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E35" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="F35" s="6" t="s">
-        <v>65</v>
-      </c>
+      <c r="E35" s="6"/>
+      <c r="F35" s="6"/>
       <c r="G35" s="6"/>
-      <c r="H35" s="94"/>
+      <c r="H35" s="91"/>
       <c r="I35" s="6"/>
       <c r="J35" s="6" t="s">
         <v>1036</v>
@@ -7258,18 +7286,18 @@
     </row>
     <row r="36" spans="2:27">
       <c r="B36" s="4" t="s">
-        <v>71</v>
+        <v>1075</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>1040</v>
+        <v>1076</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>1041</v>
+        <v>1074</v>
       </c>
       <c r="E36" s="6"/>
       <c r="F36" s="6"/>
       <c r="G36" s="6"/>
-      <c r="H36" s="94"/>
+      <c r="H36" s="91"/>
       <c r="I36" s="6"/>
       <c r="J36" s="6" t="s">
         <v>1036</v>
@@ -7278,37 +7306,37 @@
     </row>
     <row r="37" spans="2:27">
       <c r="B37" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>73</v>
+        <v>1038</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>1039</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>8</v>
+        <v>996</v>
       </c>
       <c r="E37" s="6"/>
       <c r="F37" s="6"/>
       <c r="G37" s="6"/>
-      <c r="H37" s="94"/>
+      <c r="H37" s="91"/>
       <c r="I37" s="6"/>
-      <c r="J37" s="99" t="s">
+      <c r="J37" s="96" t="s">
         <v>1037</v>
       </c>
     </row>
     <row r="38" spans="2:27">
       <c r="B38" s="4" t="s">
-        <v>1042</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>1043</v>
+        <v>1077</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>1078</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>1044</v>
+        <v>6</v>
       </c>
       <c r="E38" s="6"/>
       <c r="F38" s="6"/>
       <c r="G38" s="6"/>
-      <c r="H38" s="94"/>
+      <c r="H38" s="91"/>
       <c r="I38" s="6"/>
       <c r="J38" s="6" t="s">
         <v>1036</v>
@@ -7316,37 +7344,41 @@
     </row>
     <row r="39" spans="2:27">
       <c r="B39" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>15</v>
+        <v>84</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E39" s="6"/>
       <c r="F39" s="6"/>
       <c r="G39" s="6"/>
-      <c r="H39" s="94"/>
+      <c r="H39" s="91"/>
       <c r="I39" s="6"/>
-      <c r="J39" s="6" t="s">
-        <v>1036</v>
+      <c r="J39" s="96" t="s">
+        <v>1037</v>
       </c>
     </row>
     <row r="40" spans="2:27">
       <c r="B40" s="4" t="s">
-        <v>1045</v>
-      </c>
-      <c r="C40" s="4" t="s">
-        <v>1046</v>
+        <v>85</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>96</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E40" s="6"/>
-      <c r="F40" s="6"/>
+        <v>6</v>
+      </c>
+      <c r="E40" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="F40" s="6" t="s">
+        <v>65</v>
+      </c>
       <c r="G40" s="6"/>
-      <c r="H40" s="94"/>
+      <c r="H40" s="91"/>
       <c r="I40" s="6"/>
       <c r="J40" s="6" t="s">
         <v>1036</v>
@@ -7354,62 +7386,62 @@
     </row>
     <row r="41" spans="2:27">
       <c r="B41" s="4" t="s">
-        <v>1047</v>
+        <v>71</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>72</v>
+        <v>1040</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>74</v>
+        <v>1041</v>
       </c>
       <c r="E41" s="6"/>
       <c r="F41" s="6"/>
       <c r="G41" s="6"/>
-      <c r="H41" s="94"/>
+      <c r="H41" s="91"/>
       <c r="I41" s="6"/>
       <c r="J41" s="6" t="s">
         <v>1036</v>
       </c>
-      <c r="R41" s="86" t="s">
+      <c r="R41" s="83" t="s">
         <v>1008</v>
       </c>
     </row>
     <row r="42" spans="2:27">
       <c r="B42" s="4" t="s">
-        <v>1048</v>
-      </c>
-      <c r="C42" s="3" t="s">
-        <v>1049</v>
+        <v>71</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>73</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>74</v>
+        <v>8</v>
       </c>
       <c r="E42" s="6"/>
       <c r="F42" s="6"/>
       <c r="G42" s="6"/>
-      <c r="H42" s="94"/>
+      <c r="H42" s="91"/>
       <c r="I42" s="6"/>
-      <c r="J42" s="6" t="s">
-        <v>1036</v>
-      </c>
-      <c r="R42" s="86" t="s">
+      <c r="J42" s="96" t="s">
+        <v>1037</v>
+      </c>
+      <c r="R42" s="83" t="s">
         <v>1010</v>
       </c>
     </row>
     <row r="43" spans="2:27">
       <c r="B43" s="4" t="s">
-        <v>1048</v>
-      </c>
-      <c r="C43" s="3" t="s">
-        <v>1050</v>
+        <v>1042</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>1043</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>74</v>
+        <v>1044</v>
       </c>
       <c r="E43" s="6"/>
       <c r="F43" s="6"/>
       <c r="G43" s="6"/>
-      <c r="H43" s="94"/>
+      <c r="H43" s="91"/>
       <c r="I43" s="6"/>
       <c r="J43" s="6" t="s">
         <v>1036</v>
@@ -7417,18 +7449,18 @@
     </row>
     <row r="44" spans="2:27">
       <c r="B44" s="4" t="s">
-        <v>1051</v>
-      </c>
-      <c r="C44" s="3" t="s">
-        <v>1053</v>
+        <v>86</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>15</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E44" s="6"/>
       <c r="F44" s="6"/>
       <c r="G44" s="6"/>
-      <c r="H44" s="94"/>
+      <c r="H44" s="91"/>
       <c r="I44" s="6"/>
       <c r="J44" s="6" t="s">
         <v>1036</v>
@@ -7436,23 +7468,23 @@
     </row>
     <row r="45" spans="2:27">
       <c r="B45" s="4" t="s">
-        <v>1052</v>
-      </c>
-      <c r="C45" s="3" t="s">
-        <v>1054</v>
+        <v>1045</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>1046</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>74</v>
+        <v>8</v>
       </c>
       <c r="E45" s="6"/>
       <c r="F45" s="6"/>
       <c r="G45" s="6"/>
-      <c r="H45" s="94"/>
+      <c r="H45" s="91"/>
       <c r="I45" s="6"/>
       <c r="J45" s="6" t="s">
         <v>1036</v>
       </c>
-      <c r="R45" s="86" t="s">
+      <c r="R45" s="83" t="s">
         <v>91</v>
       </c>
       <c r="S45" t="s">
@@ -7461,27 +7493,23 @@
     </row>
     <row r="46" spans="2:27">
       <c r="B46" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="C46" s="4" t="s">
-        <v>148</v>
+        <v>1047</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>72</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="E46" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="F46" s="6" t="s">
-        <v>65</v>
-      </c>
+        <v>74</v>
+      </c>
+      <c r="E46" s="6"/>
+      <c r="F46" s="6"/>
       <c r="G46" s="6"/>
-      <c r="H46" s="94"/>
+      <c r="H46" s="91"/>
       <c r="I46" s="6"/>
       <c r="J46" s="6" t="s">
         <v>1036</v>
       </c>
-      <c r="R46" s="86" t="s">
+      <c r="R46" s="83" t="s">
         <v>1009</v>
       </c>
       <c r="S46" t="s">
@@ -7490,10 +7518,10 @@
     </row>
     <row r="47" spans="2:27">
       <c r="B47" s="4" t="s">
-        <v>1055</v>
-      </c>
-      <c r="C47" s="4" t="s">
-        <v>1056</v>
+        <v>1048</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>1049</v>
       </c>
       <c r="D47" s="4" t="s">
         <v>74</v>
@@ -7501,12 +7529,12 @@
       <c r="E47" s="6"/>
       <c r="F47" s="6"/>
       <c r="G47" s="6"/>
-      <c r="H47" s="94"/>
+      <c r="H47" s="91"/>
       <c r="I47" s="6"/>
       <c r="J47" s="6" t="s">
         <v>1036</v>
       </c>
-      <c r="R47" s="86" t="s">
+      <c r="R47" s="83" t="s">
         <v>92</v>
       </c>
       <c r="S47" t="s">
@@ -7515,23 +7543,23 @@
     </row>
     <row r="48" spans="2:27">
       <c r="B48" s="4" t="s">
-        <v>1057</v>
-      </c>
-      <c r="C48" s="4" t="s">
-        <v>1058</v>
+        <v>1048</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>1050</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>1032</v>
+        <v>74</v>
       </c>
       <c r="E48" s="6"/>
       <c r="F48" s="6"/>
       <c r="G48" s="6"/>
-      <c r="H48" s="94"/>
+      <c r="H48" s="91"/>
       <c r="I48" s="6"/>
-      <c r="J48" s="99" t="s">
-        <v>1037</v>
-      </c>
-      <c r="R48" s="86" t="s">
+      <c r="J48" s="6" t="s">
+        <v>1036</v>
+      </c>
+      <c r="R48" s="83" t="s">
         <v>1011</v>
       </c>
       <c r="S48" t="s">
@@ -7540,10 +7568,10 @@
     </row>
     <row r="49" spans="2:10">
       <c r="B49" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="C49" s="7" t="s">
-        <v>17</v>
+        <v>1051</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>1053</v>
       </c>
       <c r="D49" s="4" t="s">
         <v>8</v>
@@ -7551,26 +7579,26 @@
       <c r="E49" s="6"/>
       <c r="F49" s="6"/>
       <c r="G49" s="6"/>
-      <c r="H49" s="94"/>
+      <c r="H49" s="91"/>
       <c r="I49" s="6"/>
-      <c r="J49" s="99" t="s">
-        <v>1037</v>
+      <c r="J49" s="6" t="s">
+        <v>1036</v>
       </c>
     </row>
     <row r="50" spans="2:10">
       <c r="B50" s="4" t="s">
-        <v>1065</v>
-      </c>
-      <c r="C50" s="7" t="s">
-        <v>1066</v>
+        <v>1052</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>1054</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>105</v>
+        <v>74</v>
       </c>
       <c r="E50" s="6"/>
       <c r="F50" s="6"/>
       <c r="G50" s="6"/>
-      <c r="H50" s="94"/>
+      <c r="H50" s="91"/>
       <c r="I50" s="6"/>
       <c r="J50" s="6" t="s">
         <v>1036</v>
@@ -7578,18 +7606,22 @@
     </row>
     <row r="51" spans="2:10">
       <c r="B51" s="4" t="s">
-        <v>1059</v>
-      </c>
-      <c r="C51" s="7" t="s">
-        <v>1060</v>
+        <v>146</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>148</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>1061</v>
-      </c>
-      <c r="E51" s="6"/>
-      <c r="F51" s="6"/>
+        <v>6</v>
+      </c>
+      <c r="E51" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="F51" s="6" t="s">
+        <v>65</v>
+      </c>
       <c r="G51" s="6"/>
-      <c r="H51" s="94"/>
+      <c r="H51" s="91"/>
       <c r="I51" s="6"/>
       <c r="J51" s="6" t="s">
         <v>1036</v>
@@ -7597,27 +7629,122 @@
     </row>
     <row r="52" spans="2:10">
       <c r="B52" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="C52" s="7" t="s">
-        <v>18</v>
+        <v>1055</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>1056</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>16</v>
+        <v>74</v>
       </c>
       <c r="E52" s="6"/>
       <c r="F52" s="6"/>
-      <c r="G52" s="6" t="s">
-        <v>437</v>
-      </c>
-      <c r="H52" s="94"/>
+      <c r="G52" s="6"/>
+      <c r="H52" s="91"/>
       <c r="I52" s="6"/>
       <c r="J52" s="6" t="s">
         <v>1036</v>
       </c>
     </row>
     <row r="53" spans="2:10">
-      <c r="J53" s="98"/>
+      <c r="B53" s="4" t="s">
+        <v>1057</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>1058</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>1032</v>
+      </c>
+      <c r="E53" s="6"/>
+      <c r="F53" s="6"/>
+      <c r="G53" s="6"/>
+      <c r="H53" s="91"/>
+      <c r="I53" s="6"/>
+      <c r="J53" s="96" t="s">
+        <v>1037</v>
+      </c>
+    </row>
+    <row r="54" spans="2:10">
+      <c r="B54" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C54" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E54" s="6"/>
+      <c r="F54" s="6"/>
+      <c r="G54" s="6"/>
+      <c r="H54" s="91"/>
+      <c r="I54" s="6"/>
+      <c r="J54" s="96" t="s">
+        <v>1037</v>
+      </c>
+    </row>
+    <row r="55" spans="2:10">
+      <c r="B55" s="98" t="s">
+        <v>1065</v>
+      </c>
+      <c r="C55" s="98" t="s">
+        <v>1066</v>
+      </c>
+      <c r="D55" s="98" t="s">
+        <v>105</v>
+      </c>
+      <c r="E55" s="99"/>
+      <c r="F55" s="99"/>
+      <c r="G55" s="99"/>
+      <c r="H55" s="100"/>
+      <c r="I55" s="99"/>
+      <c r="J55" s="99" t="s">
+        <v>1036</v>
+      </c>
+    </row>
+    <row r="56" spans="2:10">
+      <c r="B56" s="4" t="s">
+        <v>1059</v>
+      </c>
+      <c r="C56" s="7" t="s">
+        <v>1060</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>1061</v>
+      </c>
+      <c r="E56" s="6"/>
+      <c r="F56" s="6"/>
+      <c r="G56" s="6"/>
+      <c r="H56" s="91"/>
+      <c r="I56" s="6"/>
+      <c r="J56" s="6" t="s">
+        <v>1036</v>
+      </c>
+    </row>
+    <row r="57" spans="2:10">
+      <c r="B57" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C57" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D57" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E57" s="6"/>
+      <c r="F57" s="6"/>
+      <c r="G57" s="6" t="s">
+        <v>437</v>
+      </c>
+      <c r="H57" s="91"/>
+      <c r="I57" s="6"/>
+      <c r="J57" s="6" t="s">
+        <v>1036</v>
+      </c>
+    </row>
+    <row r="58" spans="2:10">
+      <c r="J58" s="95"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -9412,25 +9539,25 @@
       <c r="H72" s="68"/>
     </row>
     <row r="73" spans="1:8" ht="30" customHeight="1">
-      <c r="A73" s="87" t="s">
+      <c r="A73" s="84" t="s">
         <v>111</v>
       </c>
-      <c r="B73" s="89" t="s">
+      <c r="B73" s="86" t="s">
         <v>338</v>
       </c>
-      <c r="C73" s="87" t="s">
+      <c r="C73" s="84" t="s">
         <v>339</v>
       </c>
-      <c r="D73" s="87" t="s">
+      <c r="D73" s="84" t="s">
         <v>165</v>
       </c>
-      <c r="E73" s="87" t="s">
+      <c r="E73" s="84" t="s">
         <v>101</v>
       </c>
-      <c r="F73" s="87" t="s">
+      <c r="F73" s="84" t="s">
         <v>175</v>
       </c>
-      <c r="G73" s="88" t="s">
+      <c r="G73" s="85" t="s">
         <v>340</v>
       </c>
       <c r="H73" s="68" t="s">
@@ -9438,168 +9565,168 @@
       </c>
     </row>
     <row r="74" spans="1:8" ht="30" customHeight="1">
-      <c r="A74" s="87"/>
-      <c r="B74" s="89"/>
-      <c r="C74" s="87"/>
-      <c r="D74" s="87"/>
-      <c r="E74" s="87"/>
-      <c r="F74" s="87"/>
-      <c r="G74" s="88"/>
+      <c r="A74" s="84"/>
+      <c r="B74" s="86"/>
+      <c r="C74" s="84"/>
+      <c r="D74" s="84"/>
+      <c r="E74" s="84"/>
+      <c r="F74" s="84"/>
+      <c r="G74" s="85"/>
       <c r="H74" s="68" t="s">
         <v>342</v>
       </c>
     </row>
     <row r="75" spans="1:8" ht="30" customHeight="1">
-      <c r="A75" s="80" t="s">
+      <c r="A75" s="69" t="s">
         <v>107</v>
       </c>
-      <c r="B75" s="81" t="s">
+      <c r="B75" s="70" t="s">
         <v>343</v>
       </c>
-      <c r="C75" s="80" t="s">
+      <c r="C75" s="69" t="s">
         <v>344</v>
       </c>
-      <c r="D75" s="80" t="s">
+      <c r="D75" s="69" t="s">
         <v>165</v>
       </c>
-      <c r="E75" s="80" t="s">
+      <c r="E75" s="69" t="s">
         <v>101</v>
       </c>
-      <c r="F75" s="80" t="s">
+      <c r="F75" s="69" t="s">
         <v>175</v>
       </c>
-      <c r="G75" s="82" t="s">
+      <c r="G75" s="68" t="s">
         <v>345</v>
       </c>
-      <c r="H75" s="82"/>
+      <c r="H75" s="68"/>
     </row>
     <row r="76" spans="1:8" ht="30" customHeight="1">
-      <c r="A76" s="80" t="s">
+      <c r="A76" s="69" t="s">
         <v>255</v>
       </c>
-      <c r="B76" s="81" t="s">
+      <c r="B76" s="70" t="s">
         <v>346</v>
       </c>
-      <c r="C76" s="80" t="s">
+      <c r="C76" s="69" t="s">
         <v>347</v>
       </c>
-      <c r="D76" s="80" t="s">
+      <c r="D76" s="69" t="s">
         <v>165</v>
       </c>
-      <c r="E76" s="80" t="s">
+      <c r="E76" s="69" t="s">
         <v>101</v>
       </c>
-      <c r="F76" s="80" t="s">
+      <c r="F76" s="69" t="s">
         <v>166</v>
       </c>
-      <c r="G76" s="82" t="s">
+      <c r="G76" s="68" t="s">
         <v>258</v>
       </c>
-      <c r="H76" s="82" t="s">
+      <c r="H76" s="68" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="77" spans="1:8" ht="30" customHeight="1">
-      <c r="A77" s="80" t="s">
+      <c r="A77" s="69" t="s">
         <v>255</v>
       </c>
-      <c r="B77" s="81" t="s">
+      <c r="B77" s="70" t="s">
         <v>348</v>
       </c>
-      <c r="C77" s="80" t="s">
+      <c r="C77" s="69" t="s">
         <v>349</v>
       </c>
-      <c r="D77" s="80" t="s">
+      <c r="D77" s="69" t="s">
         <v>165</v>
       </c>
-      <c r="E77" s="80" t="s">
+      <c r="E77" s="69" t="s">
         <v>101</v>
       </c>
-      <c r="F77" s="80" t="s">
+      <c r="F77" s="69" t="s">
         <v>166</v>
       </c>
-      <c r="G77" s="82" t="s">
+      <c r="G77" s="68" t="s">
         <v>258</v>
       </c>
-      <c r="H77" s="82" t="s">
+      <c r="H77" s="68" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="78" spans="1:8" ht="30" customHeight="1">
-      <c r="A78" s="80" t="s">
+      <c r="A78" s="69" t="s">
         <v>255</v>
       </c>
-      <c r="B78" s="81" t="s">
+      <c r="B78" s="70" t="s">
         <v>350</v>
       </c>
-      <c r="C78" s="80" t="s">
+      <c r="C78" s="69" t="s">
         <v>351</v>
       </c>
-      <c r="D78" s="80" t="s">
+      <c r="D78" s="69" t="s">
         <v>165</v>
       </c>
-      <c r="E78" s="80" t="s">
+      <c r="E78" s="69" t="s">
         <v>101</v>
       </c>
-      <c r="F78" s="80" t="s">
+      <c r="F78" s="69" t="s">
         <v>166</v>
       </c>
-      <c r="G78" s="82" t="s">
+      <c r="G78" s="68" t="s">
         <v>258</v>
       </c>
-      <c r="H78" s="82" t="s">
+      <c r="H78" s="68" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="79" spans="1:8" ht="30" customHeight="1">
-      <c r="A79" s="80" t="s">
+      <c r="A79" s="69" t="s">
         <v>255</v>
       </c>
-      <c r="B79" s="81" t="s">
+      <c r="B79" s="70" t="s">
         <v>352</v>
       </c>
-      <c r="C79" s="80" t="s">
+      <c r="C79" s="69" t="s">
         <v>353</v>
       </c>
-      <c r="D79" s="80" t="s">
+      <c r="D79" s="69" t="s">
         <v>165</v>
       </c>
-      <c r="E79" s="80" t="s">
+      <c r="E79" s="69" t="s">
         <v>101</v>
       </c>
-      <c r="F79" s="80" t="s">
+      <c r="F79" s="69" t="s">
         <v>166</v>
       </c>
-      <c r="G79" s="82" t="s">
+      <c r="G79" s="68" t="s">
         <v>258</v>
       </c>
-      <c r="H79" s="82" t="s">
+      <c r="H79" s="68" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="80" spans="1:8" ht="30" customHeight="1">
-      <c r="A80" s="80" t="s">
+      <c r="A80" s="69" t="s">
         <v>100</v>
       </c>
-      <c r="B80" s="81" t="s">
+      <c r="B80" s="70" t="s">
         <v>354</v>
       </c>
-      <c r="C80" s="80" t="s">
+      <c r="C80" s="69" t="s">
         <v>355</v>
       </c>
-      <c r="D80" s="80" t="s">
+      <c r="D80" s="69" t="s">
         <v>165</v>
       </c>
-      <c r="E80" s="80" t="s">
+      <c r="E80" s="69" t="s">
         <v>101</v>
       </c>
-      <c r="F80" s="80" t="s">
+      <c r="F80" s="69" t="s">
         <v>166</v>
       </c>
-      <c r="G80" s="82" t="s">
+      <c r="G80" s="68" t="s">
         <v>356</v>
       </c>
-      <c r="H80" s="82"/>
+      <c r="H80" s="68"/>
     </row>
     <row r="81" spans="1:8" ht="30" customHeight="1">
       <c r="A81" s="39" t="s">
@@ -10446,11 +10573,11 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:7" ht="21" customHeight="1">
-      <c r="B2" s="90" t="s">
+      <c r="B2" s="87" t="s">
         <v>520</v>
       </c>
-      <c r="C2" s="90"/>
-      <c r="D2" s="90"/>
+      <c r="C2" s="87"/>
+      <c r="D2" s="87"/>
     </row>
     <row r="3" spans="2:7" ht="17.5" thickBot="1"/>
     <row r="4" spans="2:7" ht="21" customHeight="1" thickBot="1">
@@ -10938,10 +11065,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:7">
-      <c r="D1" s="91" t="s">
+      <c r="D1" s="88" t="s">
         <v>647</v>
       </c>
-      <c r="E1" s="91"/>
+      <c r="E1" s="88"/>
     </row>
     <row r="3" spans="2:7" ht="20.5">
       <c r="B3" s="60" t="s">
@@ -13509,7 +13636,7 @@
       <c r="C13" s="25" t="s">
         <v>818</v>
       </c>
-      <c r="E13" s="100"/>
+      <c r="E13" s="97"/>
       <c r="F13" s="25" t="s">
         <v>319</v>
       </c>

</xml_diff>

<commit_message>
Update Fishing Bots (Kkambo, Vienna, HighFishing) and Launcher
</commit_message>
<xml_diff>
--- a/낚시 오픈일.xlsx
+++ b/낚시 오픈일.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\gemini\fishing_bot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0999AAB9-D530-4342-91D9-A9E2FB69B594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7166B5B4-26A9-415B-A3A3-57EF2CD99008}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1210" yWindow="0" windowWidth="13860" windowHeight="17280" xr2:uid="{148B82DD-3426-458A-916A-D3FE202A9A2C}"/>
+    <workbookView xWindow="-165" yWindow="-165" windowWidth="29130" windowHeight="17610" activeTab="5" xr2:uid="{148B82DD-3426-458A-916A-D3FE202A9A2C}"/>
   </bookViews>
   <sheets>
     <sheet name="작성자_DK" sheetId="1" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2245" uniqueCount="1079">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2294" uniqueCount="1104">
   <si>
     <t>선사</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -4126,10 +4126,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>3월 03일(화) 12시</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>만석선단</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -4179,6 +4175,110 @@
   </si>
   <si>
     <t>크루즈호</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1월 31일(토) 18시</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>청남호</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>['1', '11', '10', '20', '2', '12', '9', '19', '3', '13', '8', '18']</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>3월 03일(화) 13시</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>조커호</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>홍원항</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>아리랑호</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>자연피싱호</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2월 01일(일) 12시</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>독수리호</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>황금백호</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>안면도</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>블루오션호</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>좌석X</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2단계</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>남당항 장현호</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>좌석O</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>대천항 팀만수호</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>삼길포항 만석호</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>맵핑O</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>맵핑X</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>자리O</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>자리X</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>구매항 악바리호</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>자리선택특이사항</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>오천항 샤크호</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -4444,7 +4544,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="18">
+  <fills count="19">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -4544,6 +4644,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -4958,21 +5064,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -4991,13 +5082,7 @@
     <xf numFmtId="0" fontId="4" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5009,8 +5094,29 @@
     <xf numFmtId="0" fontId="3" fillId="17" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -5338,14 +5444,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A39E8B7-AF51-4CA2-AF7F-525187CC5D56}">
-  <dimension ref="B2:AA58"/>
+  <dimension ref="B2:AA64"/>
   <sheetFormatPr defaultRowHeight="17"/>
   <cols>
-    <col min="1" max="1" width="3.4140625" customWidth="1"/>
+    <col min="1" max="1" width="3.33203125" customWidth="1"/>
     <col min="2" max="2" width="20.58203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" style="26" customWidth="1"/>
+    <col min="3" max="3" width="15.83203125" style="26" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="6.6640625" customWidth="1"/>
+    <col min="5" max="5" width="6.58203125" customWidth="1"/>
     <col min="6" max="6" width="8.25" customWidth="1"/>
     <col min="7" max="7" width="12.08203125" customWidth="1"/>
     <col min="8" max="8" width="8.75" customWidth="1"/>
@@ -5353,15 +5459,15 @@
     <col min="11" max="11" width="6.75" customWidth="1"/>
     <col min="12" max="12" width="4.25" customWidth="1"/>
     <col min="13" max="13" width="16.08203125" customWidth="1"/>
-    <col min="14" max="14" width="8.1640625" customWidth="1"/>
+    <col min="14" max="14" width="8.08203125" customWidth="1"/>
     <col min="15" max="15" width="11.58203125" customWidth="1"/>
-    <col min="16" max="16" width="8.9140625" customWidth="1"/>
+    <col min="16" max="16" width="8.83203125" customWidth="1"/>
     <col min="17" max="17" width="17.83203125" customWidth="1"/>
     <col min="18" max="18" width="16.5" customWidth="1"/>
     <col min="19" max="19" width="12" customWidth="1"/>
     <col min="20" max="20" width="11.75" customWidth="1"/>
-    <col min="21" max="21" width="6.9140625" customWidth="1"/>
-    <col min="22" max="22" width="9.6640625" style="16" customWidth="1"/>
+    <col min="21" max="21" width="6.83203125" customWidth="1"/>
+    <col min="22" max="22" width="9.58203125" style="16" customWidth="1"/>
     <col min="23" max="23" width="10.08203125" customWidth="1"/>
     <col min="24" max="24" width="8.25" customWidth="1"/>
     <col min="25" max="25" width="14.83203125" customWidth="1"/>
@@ -5388,7 +5494,7 @@
       <c r="G2" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="H2" s="89" t="s">
+      <c r="H2" s="84" t="s">
         <v>1034</v>
       </c>
       <c r="I2" s="1" t="s">
@@ -5462,7 +5568,7 @@
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="6"/>
-      <c r="H3" s="90" t="s">
+      <c r="H3" s="85" t="s">
         <v>78</v>
       </c>
       <c r="I3" s="2"/>
@@ -5530,7 +5636,7 @@
       <c r="G4" s="2" t="s">
         <v>764</v>
       </c>
-      <c r="H4" s="91"/>
+      <c r="H4" s="86"/>
       <c r="I4" s="6"/>
       <c r="J4" s="6" t="s">
         <v>1036</v>
@@ -5594,7 +5700,7 @@
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="6"/>
-      <c r="H5" s="91"/>
+      <c r="H5" s="86"/>
       <c r="I5" s="6"/>
       <c r="J5" s="6" t="s">
         <v>1036</v>
@@ -5662,9 +5768,9 @@
         <v>65</v>
       </c>
       <c r="G6" s="6"/>
-      <c r="H6" s="91"/>
+      <c r="H6" s="86"/>
       <c r="I6" s="6"/>
-      <c r="J6" s="96" t="s">
+      <c r="J6" s="90" t="s">
         <v>1037</v>
       </c>
       <c r="K6" s="51"/>
@@ -5718,9 +5824,9 @@
       <c r="E7" s="6"/>
       <c r="F7" s="6"/>
       <c r="G7" s="6"/>
-      <c r="H7" s="91"/>
+      <c r="H7" s="86"/>
       <c r="I7" s="6"/>
-      <c r="J7" s="96" t="s">
+      <c r="J7" s="90" t="s">
         <v>1037</v>
       </c>
       <c r="K7" s="51"/>
@@ -5782,7 +5888,7 @@
       <c r="E8" s="6"/>
       <c r="F8" s="6"/>
       <c r="G8" s="6"/>
-      <c r="H8" s="91"/>
+      <c r="H8" s="86"/>
       <c r="I8" s="6"/>
       <c r="J8" s="6" t="s">
         <v>1036</v>
@@ -5848,7 +5954,7 @@
       <c r="G9" s="6" t="s">
         <v>439</v>
       </c>
-      <c r="H9" s="91"/>
+      <c r="H9" s="86"/>
       <c r="I9" s="6" t="s">
         <v>1018</v>
       </c>
@@ -5907,7 +6013,7 @@
       <c r="B10" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="C10" s="94" t="s">
+      <c r="C10" s="89" t="s">
         <v>103</v>
       </c>
       <c r="D10" s="14" t="s">
@@ -5920,8 +6026,8 @@
       <c r="G10" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="H10" s="91"/>
-      <c r="I10" s="93" t="s">
+      <c r="H10" s="86"/>
+      <c r="I10" s="88" t="s">
         <v>1015</v>
       </c>
       <c r="J10" s="6" t="s">
@@ -5982,7 +6088,7 @@
         <v>156</v>
       </c>
       <c r="G11" s="6"/>
-      <c r="H11" s="91" t="s">
+      <c r="H11" s="86" t="s">
         <v>78</v>
       </c>
       <c r="I11" s="6"/>
@@ -6058,9 +6164,9 @@
       <c r="G12" s="6" t="s">
         <v>437</v>
       </c>
-      <c r="H12" s="91"/>
+      <c r="H12" s="86"/>
       <c r="I12" s="6"/>
-      <c r="J12" s="96" t="s">
+      <c r="J12" s="90" t="s">
         <v>1037</v>
       </c>
       <c r="K12" s="51"/>
@@ -6113,7 +6219,7 @@
       <c r="B13" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="C13" s="94" t="s">
+      <c r="C13" s="89" t="s">
         <v>9</v>
       </c>
       <c r="D13" s="14" t="s">
@@ -6124,8 +6230,8 @@
         <v>152</v>
       </c>
       <c r="G13" s="6"/>
-      <c r="H13" s="91"/>
-      <c r="I13" s="93" t="s">
+      <c r="H13" s="86"/>
+      <c r="I13" s="88" t="s">
         <v>1018</v>
       </c>
       <c r="J13" s="6" t="s">
@@ -6194,7 +6300,7 @@
       <c r="G14" s="6" t="s">
         <v>438</v>
       </c>
-      <c r="H14" s="91"/>
+      <c r="H14" s="86"/>
       <c r="I14" s="6"/>
       <c r="J14" s="6" t="s">
         <v>1036</v>
@@ -6258,7 +6364,7 @@
       <c r="E15" s="6"/>
       <c r="F15" s="6"/>
       <c r="G15" s="6"/>
-      <c r="H15" s="91"/>
+      <c r="H15" s="86"/>
       <c r="I15" s="6"/>
       <c r="J15" s="6" t="s">
         <v>1036</v>
@@ -6300,9 +6406,9 @@
       <c r="G16" s="6" t="s">
         <v>437</v>
       </c>
-      <c r="H16" s="91"/>
+      <c r="H16" s="86"/>
       <c r="I16" s="6"/>
-      <c r="J16" s="96" t="s">
+      <c r="J16" s="90" t="s">
         <v>1037</v>
       </c>
       <c r="K16" s="51"/>
@@ -6360,7 +6466,7 @@
         <v>449</v>
       </c>
       <c r="G17" s="6"/>
-      <c r="H17" s="91" t="s">
+      <c r="H17" s="86" t="s">
         <v>78</v>
       </c>
       <c r="I17" s="6"/>
@@ -6420,9 +6526,9 @@
         <v>449</v>
       </c>
       <c r="G18" s="6"/>
-      <c r="H18" s="91"/>
+      <c r="H18" s="86"/>
       <c r="I18" s="6"/>
-      <c r="J18" s="96" t="s">
+      <c r="J18" s="90" t="s">
         <v>1037</v>
       </c>
       <c r="K18" s="51"/>
@@ -6478,7 +6584,7 @@
       <c r="G19" s="57" t="s">
         <v>524</v>
       </c>
-      <c r="H19" s="92"/>
+      <c r="H19" s="87"/>
       <c r="I19" s="57"/>
       <c r="J19" s="6" t="s">
         <v>1036</v>
@@ -6548,7 +6654,7 @@
         <v>449</v>
       </c>
       <c r="G20" s="6"/>
-      <c r="H20" s="91"/>
+      <c r="H20" s="86"/>
       <c r="I20" s="6"/>
       <c r="J20" s="6" t="s">
         <v>1036</v>
@@ -6606,7 +6712,7 @@
         <v>431</v>
       </c>
       <c r="G21" s="6"/>
-      <c r="H21" s="91"/>
+      <c r="H21" s="86"/>
       <c r="I21" s="6"/>
       <c r="J21" s="6" t="s">
         <v>1036</v>
@@ -6664,7 +6770,7 @@
         <v>449</v>
       </c>
       <c r="G22" s="6"/>
-      <c r="H22" s="91" t="s">
+      <c r="H22" s="86" t="s">
         <v>58</v>
       </c>
       <c r="I22" s="6"/>
@@ -6724,7 +6830,7 @@
       <c r="G23" s="2" t="s">
         <v>764</v>
       </c>
-      <c r="H23" s="91"/>
+      <c r="H23" s="86"/>
       <c r="I23" s="6"/>
       <c r="J23" s="6" t="s">
         <v>1036</v>
@@ -6782,7 +6888,7 @@
         <v>65</v>
       </c>
       <c r="G24" s="6"/>
-      <c r="H24" s="91"/>
+      <c r="H24" s="86"/>
       <c r="I24" s="6"/>
       <c r="J24" s="6" t="s">
         <v>1036</v>
@@ -6844,8 +6950,8 @@
       <c r="G25" s="6" t="s">
         <v>761</v>
       </c>
-      <c r="H25" s="91"/>
-      <c r="I25" s="101" t="s">
+      <c r="H25" s="86"/>
+      <c r="I25" s="6" t="s">
         <v>1017</v>
       </c>
       <c r="J25" s="6" t="s">
@@ -6906,9 +7012,9 @@
       <c r="G26" s="6" t="s">
         <v>990</v>
       </c>
-      <c r="H26" s="91"/>
+      <c r="H26" s="86"/>
       <c r="I26" s="6" t="s">
-        <v>1067</v>
+        <v>1066</v>
       </c>
       <c r="J26" s="6" t="s">
         <v>1036</v>
@@ -6936,7 +7042,7 @@
         <v>65</v>
       </c>
       <c r="G27" s="6"/>
-      <c r="H27" s="91"/>
+      <c r="H27" s="86"/>
       <c r="I27" s="6"/>
       <c r="J27" s="6" t="s">
         <v>1036</v>
@@ -6948,19 +7054,19 @@
       <c r="AA27" s="16"/>
     </row>
     <row r="28" spans="2:27">
-      <c r="B28" s="4" t="s">
+      <c r="B28" s="14" t="s">
         <v>1022</v>
       </c>
-      <c r="C28" s="3" t="s">
+      <c r="C28" s="14" t="s">
         <v>1023</v>
       </c>
-      <c r="D28" s="4" t="s">
+      <c r="D28" s="14" t="s">
         <v>1024</v>
       </c>
       <c r="E28" s="6"/>
       <c r="F28" s="6"/>
       <c r="G28" s="6"/>
-      <c r="H28" s="91"/>
+      <c r="H28" s="86"/>
       <c r="I28" s="6"/>
       <c r="J28" s="6" t="s">
         <v>1036</v>
@@ -6976,19 +7082,19 @@
       <c r="AA28" s="16"/>
     </row>
     <row r="29" spans="2:27">
-      <c r="B29" s="4" t="s">
+      <c r="B29" s="14" t="s">
         <v>1025</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="C29" s="14" t="s">
         <v>1026</v>
       </c>
-      <c r="D29" s="4" t="s">
+      <c r="D29" s="14" t="s">
         <v>8</v>
       </c>
       <c r="E29" s="6"/>
       <c r="F29" s="6"/>
       <c r="G29" s="6"/>
-      <c r="H29" s="91"/>
+      <c r="H29" s="86"/>
       <c r="I29" s="6"/>
       <c r="J29" s="6" t="s">
         <v>1036</v>
@@ -7000,19 +7106,19 @@
       <c r="AA29" s="16"/>
     </row>
     <row r="30" spans="2:27">
-      <c r="B30" s="4" t="s">
+      <c r="B30" s="14" t="s">
+        <v>1067</v>
+      </c>
+      <c r="C30" s="14" t="s">
         <v>1068</v>
       </c>
-      <c r="C30" s="3" t="s">
-        <v>1069</v>
-      </c>
-      <c r="D30" s="4" t="s">
+      <c r="D30" s="14" t="s">
         <v>6</v>
       </c>
       <c r="E30" s="6"/>
       <c r="F30" s="6"/>
       <c r="G30" s="6"/>
-      <c r="H30" s="91"/>
+      <c r="H30" s="86"/>
       <c r="I30" s="6"/>
       <c r="J30" s="6" t="s">
         <v>1036</v>
@@ -7023,19 +7129,19 @@
       <c r="AA30" s="16"/>
     </row>
     <row r="31" spans="2:27" ht="17.5" thickBot="1">
-      <c r="B31" s="4" t="s">
-        <v>1028</v>
-      </c>
-      <c r="C31" s="3" t="s">
-        <v>1030</v>
-      </c>
-      <c r="D31" s="4" t="s">
-        <v>1032</v>
+      <c r="B31" s="14" t="s">
+        <v>1078</v>
+      </c>
+      <c r="C31" s="14" t="s">
+        <v>1079</v>
+      </c>
+      <c r="D31" s="14" t="s">
+        <v>11</v>
       </c>
       <c r="E31" s="6"/>
       <c r="F31" s="6"/>
       <c r="G31" s="6"/>
-      <c r="H31" s="91"/>
+      <c r="H31" s="86"/>
       <c r="I31" s="6"/>
       <c r="J31" s="6" t="s">
         <v>1036</v>
@@ -7086,22 +7192,22 @@
       </c>
     </row>
     <row r="32" spans="2:27" ht="17.5" thickTop="1">
-      <c r="B32" s="4" t="s">
-        <v>1029</v>
-      </c>
-      <c r="C32" s="3" t="s">
-        <v>1031</v>
-      </c>
-      <c r="D32" s="4" t="s">
-        <v>523</v>
+      <c r="B32" s="14" t="s">
+        <v>1028</v>
+      </c>
+      <c r="C32" s="14" t="s">
+        <v>1030</v>
+      </c>
+      <c r="D32" s="14" t="s">
+        <v>1032</v>
       </c>
       <c r="E32" s="6"/>
       <c r="F32" s="6"/>
       <c r="G32" s="6"/>
-      <c r="H32" s="91"/>
+      <c r="H32" s="86"/>
       <c r="I32" s="6"/>
-      <c r="J32" s="96" t="s">
-        <v>1037</v>
+      <c r="J32" s="6" t="s">
+        <v>1036</v>
       </c>
       <c r="K32" s="51"/>
       <c r="M32" s="20" t="s">
@@ -7145,22 +7251,22 @@
       <c r="AA32" s="24"/>
     </row>
     <row r="33" spans="2:27">
-      <c r="B33" s="4" t="s">
-        <v>991</v>
-      </c>
-      <c r="C33" s="3" t="s">
-        <v>992</v>
-      </c>
-      <c r="D33" s="4" t="s">
-        <v>6</v>
+      <c r="B33" s="14" t="s">
+        <v>1029</v>
+      </c>
+      <c r="C33" s="14" t="s">
+        <v>1031</v>
+      </c>
+      <c r="D33" s="14" t="s">
+        <v>523</v>
       </c>
       <c r="E33" s="6"/>
       <c r="F33" s="6"/>
       <c r="G33" s="6"/>
-      <c r="H33" s="91"/>
+      <c r="H33" s="86"/>
       <c r="I33" s="6"/>
-      <c r="J33" s="6" t="s">
-        <v>1036</v>
+      <c r="J33" s="90" t="s">
+        <v>1037</v>
       </c>
       <c r="K33" s="51"/>
       <c r="M33" s="7" t="s">
@@ -7206,22 +7312,22 @@
       </c>
     </row>
     <row r="34" spans="2:27">
-      <c r="B34" s="4" t="s">
-        <v>1070</v>
-      </c>
-      <c r="C34" s="3" t="s">
-        <v>1071</v>
-      </c>
-      <c r="D34" s="4" t="s">
-        <v>1074</v>
+      <c r="B34" s="14" t="s">
+        <v>991</v>
+      </c>
+      <c r="C34" s="14" t="s">
+        <v>1084</v>
+      </c>
+      <c r="D34" s="14" t="s">
+        <v>8</v>
       </c>
       <c r="E34" s="6"/>
       <c r="F34" s="6"/>
       <c r="G34" s="6"/>
-      <c r="H34" s="91"/>
+      <c r="H34" s="86"/>
       <c r="I34" s="6"/>
-      <c r="J34" s="6" t="s">
-        <v>1036</v>
+      <c r="J34" s="90" t="s">
+        <v>1037</v>
       </c>
       <c r="K34" s="51"/>
       <c r="M34" s="18" t="s">
@@ -7265,19 +7371,19 @@
       <c r="AA34" s="19"/>
     </row>
     <row r="35" spans="2:27">
-      <c r="B35" s="4" t="s">
-        <v>1072</v>
-      </c>
-      <c r="C35" s="3" t="s">
-        <v>1073</v>
-      </c>
-      <c r="D35" s="4" t="s">
+      <c r="B35" s="14" t="s">
+        <v>991</v>
+      </c>
+      <c r="C35" s="14" t="s">
+        <v>992</v>
+      </c>
+      <c r="D35" s="14" t="s">
         <v>6</v>
       </c>
       <c r="E35" s="6"/>
       <c r="F35" s="6"/>
       <c r="G35" s="6"/>
-      <c r="H35" s="91"/>
+      <c r="H35" s="86"/>
       <c r="I35" s="6"/>
       <c r="J35" s="6" t="s">
         <v>1036</v>
@@ -7285,19 +7391,19 @@
       <c r="K35" s="51"/>
     </row>
     <row r="36" spans="2:27">
-      <c r="B36" s="4" t="s">
-        <v>1075</v>
-      </c>
-      <c r="C36" s="3" t="s">
-        <v>1076</v>
-      </c>
-      <c r="D36" s="4" t="s">
-        <v>1074</v>
+      <c r="B36" s="14" t="s">
+        <v>1069</v>
+      </c>
+      <c r="C36" s="14" t="s">
+        <v>1070</v>
+      </c>
+      <c r="D36" s="14" t="s">
+        <v>1073</v>
       </c>
       <c r="E36" s="6"/>
       <c r="F36" s="6"/>
       <c r="G36" s="6"/>
-      <c r="H36" s="91"/>
+      <c r="H36" s="86"/>
       <c r="I36" s="6"/>
       <c r="J36" s="6" t="s">
         <v>1036</v>
@@ -7305,99 +7411,95 @@
       <c r="K36" s="51"/>
     </row>
     <row r="37" spans="2:27">
-      <c r="B37" s="4" t="s">
-        <v>1038</v>
-      </c>
-      <c r="C37" s="3" t="s">
-        <v>1039</v>
-      </c>
-      <c r="D37" s="4" t="s">
-        <v>996</v>
+      <c r="B37" s="14" t="s">
+        <v>1071</v>
+      </c>
+      <c r="C37" s="14" t="s">
+        <v>1072</v>
+      </c>
+      <c r="D37" s="14" t="s">
+        <v>6</v>
       </c>
       <c r="E37" s="6"/>
       <c r="F37" s="6"/>
       <c r="G37" s="6"/>
-      <c r="H37" s="91"/>
+      <c r="H37" s="86"/>
       <c r="I37" s="6"/>
-      <c r="J37" s="96" t="s">
-        <v>1037</v>
+      <c r="J37" s="6" t="s">
+        <v>1036</v>
       </c>
     </row>
     <row r="38" spans="2:27">
-      <c r="B38" s="4" t="s">
-        <v>1077</v>
-      </c>
-      <c r="C38" s="3" t="s">
-        <v>1078</v>
-      </c>
-      <c r="D38" s="4" t="s">
-        <v>6</v>
+      <c r="B38" s="14" t="s">
+        <v>1074</v>
+      </c>
+      <c r="C38" s="14" t="s">
+        <v>1075</v>
+      </c>
+      <c r="D38" s="14" t="s">
+        <v>1073</v>
       </c>
       <c r="E38" s="6"/>
       <c r="F38" s="6"/>
       <c r="G38" s="6"/>
-      <c r="H38" s="91"/>
+      <c r="H38" s="86"/>
       <c r="I38" s="6"/>
       <c r="J38" s="6" t="s">
         <v>1036</v>
       </c>
     </row>
     <row r="39" spans="2:27">
-      <c r="B39" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="C39" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="D39" s="4" t="s">
-        <v>8</v>
+      <c r="B39" s="14" t="s">
+        <v>1038</v>
+      </c>
+      <c r="C39" s="14" t="s">
+        <v>1039</v>
+      </c>
+      <c r="D39" s="14" t="s">
+        <v>996</v>
       </c>
       <c r="E39" s="6"/>
       <c r="F39" s="6"/>
       <c r="G39" s="6"/>
-      <c r="H39" s="91"/>
+      <c r="H39" s="86"/>
       <c r="I39" s="6"/>
-      <c r="J39" s="96" t="s">
+      <c r="J39" s="90" t="s">
         <v>1037</v>
       </c>
     </row>
     <row r="40" spans="2:27">
-      <c r="B40" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="C40" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="D40" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="E40" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="F40" s="6" t="s">
-        <v>65</v>
-      </c>
+      <c r="B40" s="14" t="s">
+        <v>1038</v>
+      </c>
+      <c r="C40" s="14" t="s">
+        <v>1085</v>
+      </c>
+      <c r="D40" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="E40" s="6"/>
+      <c r="F40" s="6"/>
       <c r="G40" s="6"/>
-      <c r="H40" s="91"/>
+      <c r="H40" s="86"/>
       <c r="I40" s="6"/>
-      <c r="J40" s="6" t="s">
-        <v>1036</v>
+      <c r="J40" s="90" t="s">
+        <v>1037</v>
       </c>
     </row>
     <row r="41" spans="2:27">
-      <c r="B41" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="C41" s="3" t="s">
-        <v>1040</v>
-      </c>
-      <c r="D41" s="4" t="s">
-        <v>1041</v>
+      <c r="B41" s="14" t="s">
+        <v>1038</v>
+      </c>
+      <c r="C41" s="14" t="s">
+        <v>1090</v>
+      </c>
+      <c r="D41" s="14" t="s">
+        <v>436</v>
       </c>
       <c r="E41" s="6"/>
       <c r="F41" s="6"/>
       <c r="G41" s="6"/>
-      <c r="H41" s="91"/>
+      <c r="H41" s="86"/>
       <c r="I41" s="6"/>
       <c r="J41" s="6" t="s">
         <v>1036</v>
@@ -7407,79 +7509,83 @@
       </c>
     </row>
     <row r="42" spans="2:27">
-      <c r="B42" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="C42" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="D42" s="4" t="s">
-        <v>8</v>
+      <c r="B42" s="14" t="s">
+        <v>1076</v>
+      </c>
+      <c r="C42" s="14" t="s">
+        <v>1077</v>
+      </c>
+      <c r="D42" s="14" t="s">
+        <v>6</v>
       </c>
       <c r="E42" s="6"/>
       <c r="F42" s="6"/>
       <c r="G42" s="6"/>
-      <c r="H42" s="91"/>
+      <c r="H42" s="86"/>
       <c r="I42" s="6"/>
-      <c r="J42" s="96" t="s">
-        <v>1037</v>
+      <c r="J42" s="6" t="s">
+        <v>1036</v>
       </c>
       <c r="R42" s="83" t="s">
         <v>1010</v>
       </c>
     </row>
     <row r="43" spans="2:27">
-      <c r="B43" s="4" t="s">
-        <v>1042</v>
-      </c>
-      <c r="C43" s="4" t="s">
-        <v>1043</v>
-      </c>
-      <c r="D43" s="4" t="s">
-        <v>1044</v>
+      <c r="B43" s="14" t="s">
+        <v>1086</v>
+      </c>
+      <c r="C43" s="14" t="s">
+        <v>1087</v>
+      </c>
+      <c r="D43" s="14" t="s">
+        <v>8</v>
       </c>
       <c r="E43" s="6"/>
       <c r="F43" s="6"/>
       <c r="G43" s="6"/>
-      <c r="H43" s="91"/>
+      <c r="H43" s="86"/>
       <c r="I43" s="6"/>
       <c r="J43" s="6" t="s">
         <v>1036</v>
       </c>
     </row>
     <row r="44" spans="2:27">
-      <c r="B44" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="C44" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="D44" s="4" t="s">
-        <v>16</v>
+      <c r="B44" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="C44" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="D44" s="14" t="s">
+        <v>8</v>
       </c>
       <c r="E44" s="6"/>
       <c r="F44" s="6"/>
       <c r="G44" s="6"/>
-      <c r="H44" s="91"/>
+      <c r="H44" s="86"/>
       <c r="I44" s="6"/>
-      <c r="J44" s="6" t="s">
-        <v>1036</v>
+      <c r="J44" s="90" t="s">
+        <v>1037</v>
       </c>
     </row>
     <row r="45" spans="2:27">
-      <c r="B45" s="4" t="s">
-        <v>1045</v>
-      </c>
-      <c r="C45" s="4" t="s">
-        <v>1046</v>
-      </c>
-      <c r="D45" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E45" s="6"/>
-      <c r="F45" s="6"/>
+      <c r="B45" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="C45" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="D45" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="E45" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="F45" s="6" t="s">
+        <v>65</v>
+      </c>
       <c r="G45" s="6"/>
-      <c r="H45" s="91"/>
+      <c r="H45" s="86"/>
       <c r="I45" s="6"/>
       <c r="J45" s="6" t="s">
         <v>1036</v>
@@ -7492,22 +7598,22 @@
       </c>
     </row>
     <row r="46" spans="2:27">
-      <c r="B46" s="4" t="s">
-        <v>1047</v>
-      </c>
-      <c r="C46" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="D46" s="4" t="s">
-        <v>74</v>
+      <c r="B46" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="C46" s="14" t="s">
+        <v>1088</v>
+      </c>
+      <c r="D46" s="14" t="s">
+        <v>1089</v>
       </c>
       <c r="E46" s="6"/>
       <c r="F46" s="6"/>
       <c r="G46" s="6"/>
-      <c r="H46" s="91"/>
+      <c r="H46" s="86"/>
       <c r="I46" s="6"/>
-      <c r="J46" s="6" t="s">
-        <v>1036</v>
+      <c r="J46" s="90" t="s">
+        <v>1037</v>
       </c>
       <c r="R46" s="83" t="s">
         <v>1009</v>
@@ -7517,19 +7623,19 @@
       </c>
     </row>
     <row r="47" spans="2:27">
-      <c r="B47" s="4" t="s">
-        <v>1048</v>
-      </c>
-      <c r="C47" s="3" t="s">
-        <v>1049</v>
-      </c>
-      <c r="D47" s="4" t="s">
-        <v>74</v>
+      <c r="B47" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="C47" s="14" t="s">
+        <v>1040</v>
+      </c>
+      <c r="D47" s="14" t="s">
+        <v>1041</v>
       </c>
       <c r="E47" s="6"/>
       <c r="F47" s="6"/>
       <c r="G47" s="6"/>
-      <c r="H47" s="91"/>
+      <c r="H47" s="86"/>
       <c r="I47" s="6"/>
       <c r="J47" s="6" t="s">
         <v>1036</v>
@@ -7542,22 +7648,22 @@
       </c>
     </row>
     <row r="48" spans="2:27">
-      <c r="B48" s="4" t="s">
-        <v>1048</v>
-      </c>
-      <c r="C48" s="3" t="s">
-        <v>1050</v>
-      </c>
-      <c r="D48" s="4" t="s">
-        <v>74</v>
+      <c r="B48" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="C48" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="D48" s="14" t="s">
+        <v>8</v>
       </c>
       <c r="E48" s="6"/>
       <c r="F48" s="6"/>
       <c r="G48" s="6"/>
-      <c r="H48" s="91"/>
+      <c r="H48" s="86"/>
       <c r="I48" s="6"/>
-      <c r="J48" s="6" t="s">
-        <v>1036</v>
+      <c r="J48" s="90" t="s">
+        <v>1037</v>
       </c>
       <c r="R48" s="83" t="s">
         <v>1011</v>
@@ -7567,38 +7673,38 @@
       </c>
     </row>
     <row r="49" spans="2:10">
-      <c r="B49" s="4" t="s">
-        <v>1051</v>
-      </c>
-      <c r="C49" s="3" t="s">
-        <v>1053</v>
-      </c>
-      <c r="D49" s="4" t="s">
-        <v>8</v>
+      <c r="B49" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="C49" s="14" t="s">
+        <v>1082</v>
+      </c>
+      <c r="D49" s="14" t="s">
+        <v>1083</v>
       </c>
       <c r="E49" s="6"/>
       <c r="F49" s="6"/>
       <c r="G49" s="6"/>
-      <c r="H49" s="91"/>
+      <c r="H49" s="86"/>
       <c r="I49" s="6"/>
       <c r="J49" s="6" t="s">
         <v>1036</v>
       </c>
     </row>
     <row r="50" spans="2:10">
-      <c r="B50" s="4" t="s">
-        <v>1052</v>
-      </c>
-      <c r="C50" s="3" t="s">
-        <v>1054</v>
-      </c>
-      <c r="D50" s="4" t="s">
-        <v>74</v>
+      <c r="B50" s="14" t="s">
+        <v>1042</v>
+      </c>
+      <c r="C50" s="14" t="s">
+        <v>1043</v>
+      </c>
+      <c r="D50" s="14" t="s">
+        <v>1044</v>
       </c>
       <c r="E50" s="6"/>
       <c r="F50" s="6"/>
       <c r="G50" s="6"/>
-      <c r="H50" s="91"/>
+      <c r="H50" s="86"/>
       <c r="I50" s="6"/>
       <c r="J50" s="6" t="s">
         <v>1036</v>
@@ -7606,22 +7712,18 @@
     </row>
     <row r="51" spans="2:10">
       <c r="B51" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="C51" s="4" t="s">
-        <v>148</v>
+        <v>86</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="E51" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="F51" s="6" t="s">
-        <v>65</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="E51" s="6"/>
+      <c r="F51" s="6"/>
       <c r="G51" s="6"/>
-      <c r="H51" s="91"/>
+      <c r="H51" s="86"/>
       <c r="I51" s="6"/>
       <c r="J51" s="6" t="s">
         <v>1036</v>
@@ -7629,18 +7731,18 @@
     </row>
     <row r="52" spans="2:10">
       <c r="B52" s="4" t="s">
-        <v>1055</v>
-      </c>
-      <c r="C52" s="4" t="s">
-        <v>1056</v>
+        <v>1045</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>1046</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>74</v>
+        <v>8</v>
       </c>
       <c r="E52" s="6"/>
       <c r="F52" s="6"/>
       <c r="G52" s="6"/>
-      <c r="H52" s="91"/>
+      <c r="H52" s="86"/>
       <c r="I52" s="6"/>
       <c r="J52" s="6" t="s">
         <v>1036</v>
@@ -7648,75 +7750,75 @@
     </row>
     <row r="53" spans="2:10">
       <c r="B53" s="4" t="s">
-        <v>1057</v>
-      </c>
-      <c r="C53" s="4" t="s">
-        <v>1058</v>
+        <v>1047</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>72</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>1032</v>
+        <v>74</v>
       </c>
       <c r="E53" s="6"/>
       <c r="F53" s="6"/>
       <c r="G53" s="6"/>
-      <c r="H53" s="91"/>
+      <c r="H53" s="86"/>
       <c r="I53" s="6"/>
-      <c r="J53" s="96" t="s">
-        <v>1037</v>
+      <c r="J53" s="6" t="s">
+        <v>1036</v>
       </c>
     </row>
     <row r="54" spans="2:10">
       <c r="B54" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="C54" s="7" t="s">
-        <v>17</v>
+        <v>1048</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>1049</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>8</v>
+        <v>74</v>
       </c>
       <c r="E54" s="6"/>
       <c r="F54" s="6"/>
       <c r="G54" s="6"/>
-      <c r="H54" s="91"/>
+      <c r="H54" s="86"/>
       <c r="I54" s="6"/>
-      <c r="J54" s="96" t="s">
-        <v>1037</v>
+      <c r="J54" s="6" t="s">
+        <v>1036</v>
       </c>
     </row>
     <row r="55" spans="2:10">
-      <c r="B55" s="98" t="s">
-        <v>1065</v>
-      </c>
-      <c r="C55" s="98" t="s">
-        <v>1066</v>
-      </c>
-      <c r="D55" s="98" t="s">
-        <v>105</v>
-      </c>
-      <c r="E55" s="99"/>
-      <c r="F55" s="99"/>
-      <c r="G55" s="99"/>
-      <c r="H55" s="100"/>
-      <c r="I55" s="99"/>
-      <c r="J55" s="99" t="s">
+      <c r="B55" s="4" t="s">
+        <v>1048</v>
+      </c>
+      <c r="C55" s="3" t="s">
+        <v>1050</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E55" s="6"/>
+      <c r="F55" s="6"/>
+      <c r="G55" s="6"/>
+      <c r="H55" s="86"/>
+      <c r="I55" s="6"/>
+      <c r="J55" s="6" t="s">
         <v>1036</v>
       </c>
     </row>
     <row r="56" spans="2:10">
       <c r="B56" s="4" t="s">
-        <v>1059</v>
-      </c>
-      <c r="C56" s="7" t="s">
-        <v>1060</v>
+        <v>1051</v>
+      </c>
+      <c r="C56" s="3" t="s">
+        <v>1053</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>1061</v>
+        <v>8</v>
       </c>
       <c r="E56" s="6"/>
       <c r="F56" s="6"/>
       <c r="G56" s="6"/>
-      <c r="H56" s="91"/>
+      <c r="H56" s="86"/>
       <c r="I56" s="6"/>
       <c r="J56" s="6" t="s">
         <v>1036</v>
@@ -7724,27 +7826,161 @@
     </row>
     <row r="57" spans="2:10">
       <c r="B57" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="C57" s="7" t="s">
-        <v>18</v>
+        <v>1052</v>
+      </c>
+      <c r="C57" s="3" t="s">
+        <v>1054</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>16</v>
+        <v>74</v>
       </c>
       <c r="E57" s="6"/>
       <c r="F57" s="6"/>
-      <c r="G57" s="6" t="s">
-        <v>437</v>
-      </c>
-      <c r="H57" s="91"/>
+      <c r="G57" s="6"/>
+      <c r="H57" s="86"/>
       <c r="I57" s="6"/>
       <c r="J57" s="6" t="s">
         <v>1036</v>
       </c>
     </row>
     <row r="58" spans="2:10">
-      <c r="J58" s="95"/>
+      <c r="B58" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="C58" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="D58" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E58" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="F58" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="G58" s="6"/>
+      <c r="H58" s="86"/>
+      <c r="I58" s="6"/>
+      <c r="J58" s="6" t="s">
+        <v>1036</v>
+      </c>
+    </row>
+    <row r="59" spans="2:10">
+      <c r="B59" s="4" t="s">
+        <v>1055</v>
+      </c>
+      <c r="C59" s="3" t="s">
+        <v>1056</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E59" s="6"/>
+      <c r="F59" s="6"/>
+      <c r="G59" s="6"/>
+      <c r="H59" s="86"/>
+      <c r="I59" s="6"/>
+      <c r="J59" s="6" t="s">
+        <v>1036</v>
+      </c>
+    </row>
+    <row r="60" spans="2:10">
+      <c r="B60" s="4" t="s">
+        <v>1057</v>
+      </c>
+      <c r="C60" s="3" t="s">
+        <v>1058</v>
+      </c>
+      <c r="D60" s="4" t="s">
+        <v>1032</v>
+      </c>
+      <c r="E60" s="6"/>
+      <c r="F60" s="6"/>
+      <c r="G60" s="6"/>
+      <c r="H60" s="86"/>
+      <c r="I60" s="6"/>
+      <c r="J60" s="90" t="s">
+        <v>1037</v>
+      </c>
+    </row>
+    <row r="61" spans="2:10">
+      <c r="B61" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C61" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D61" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E61" s="6"/>
+      <c r="F61" s="6"/>
+      <c r="G61" s="6"/>
+      <c r="H61" s="86"/>
+      <c r="I61" s="6"/>
+      <c r="J61" s="90" t="s">
+        <v>1037</v>
+      </c>
+    </row>
+    <row r="62" spans="2:10">
+      <c r="B62" s="91" t="s">
+        <v>1081</v>
+      </c>
+      <c r="C62" s="91" t="s">
+        <v>1065</v>
+      </c>
+      <c r="D62" s="91" t="s">
+        <v>105</v>
+      </c>
+      <c r="E62" s="92"/>
+      <c r="F62" s="92"/>
+      <c r="G62" s="92"/>
+      <c r="H62" s="93"/>
+      <c r="I62" s="92"/>
+      <c r="J62" s="92" t="s">
+        <v>1036</v>
+      </c>
+    </row>
+    <row r="63" spans="2:10">
+      <c r="B63" s="4" t="s">
+        <v>1059</v>
+      </c>
+      <c r="C63" s="3" t="s">
+        <v>1060</v>
+      </c>
+      <c r="D63" s="4" t="s">
+        <v>1061</v>
+      </c>
+      <c r="E63" s="6"/>
+      <c r="F63" s="6"/>
+      <c r="G63" s="6"/>
+      <c r="H63" s="86"/>
+      <c r="I63" s="6"/>
+      <c r="J63" s="6" t="s">
+        <v>1036</v>
+      </c>
+    </row>
+    <row r="64" spans="2:10">
+      <c r="B64" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C64" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D64" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E64" s="6"/>
+      <c r="F64" s="6"/>
+      <c r="G64" s="6" t="s">
+        <v>437</v>
+      </c>
+      <c r="H64" s="86"/>
+      <c r="I64" s="6"/>
+      <c r="J64" s="6" t="s">
+        <v>1036</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -7758,10 +7994,10 @@
   <sheetFormatPr defaultRowHeight="17"/>
   <cols>
     <col min="1" max="2" width="13.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.6640625" customWidth="1"/>
+    <col min="3" max="3" width="18.58203125" customWidth="1"/>
     <col min="4" max="6" width="13.83203125" customWidth="1"/>
     <col min="7" max="7" width="71.5" customWidth="1"/>
-    <col min="8" max="8" width="58.4140625" customWidth="1"/>
+    <col min="8" max="8" width="58.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="45" customHeight="1">
@@ -9539,25 +9775,25 @@
       <c r="H72" s="68"/>
     </row>
     <row r="73" spans="1:8" ht="30" customHeight="1">
-      <c r="A73" s="84" t="s">
+      <c r="A73" s="94" t="s">
         <v>111</v>
       </c>
-      <c r="B73" s="86" t="s">
+      <c r="B73" s="96" t="s">
         <v>338</v>
       </c>
-      <c r="C73" s="84" t="s">
+      <c r="C73" s="94" t="s">
         <v>339</v>
       </c>
-      <c r="D73" s="84" t="s">
+      <c r="D73" s="94" t="s">
         <v>165</v>
       </c>
-      <c r="E73" s="84" t="s">
+      <c r="E73" s="94" t="s">
         <v>101</v>
       </c>
-      <c r="F73" s="84" t="s">
+      <c r="F73" s="94" t="s">
         <v>175</v>
       </c>
-      <c r="G73" s="85" t="s">
+      <c r="G73" s="95" t="s">
         <v>340</v>
       </c>
       <c r="H73" s="68" t="s">
@@ -9565,13 +9801,13 @@
       </c>
     </row>
     <row r="74" spans="1:8" ht="30" customHeight="1">
-      <c r="A74" s="84"/>
-      <c r="B74" s="86"/>
-      <c r="C74" s="84"/>
-      <c r="D74" s="84"/>
-      <c r="E74" s="84"/>
-      <c r="F74" s="84"/>
-      <c r="G74" s="85"/>
+      <c r="A74" s="94"/>
+      <c r="B74" s="96"/>
+      <c r="C74" s="94"/>
+      <c r="D74" s="94"/>
+      <c r="E74" s="94"/>
+      <c r="F74" s="94"/>
+      <c r="G74" s="95"/>
       <c r="H74" s="68" t="s">
         <v>342</v>
       </c>
@@ -10569,15 +10805,15 @@
     <col min="2" max="2" width="16.08203125" customWidth="1"/>
     <col min="3" max="3" width="6.75" customWidth="1"/>
     <col min="4" max="4" width="35.75" customWidth="1"/>
-    <col min="5" max="7" width="11.1640625" customWidth="1"/>
+    <col min="5" max="7" width="11.08203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:7" ht="21" customHeight="1">
-      <c r="B2" s="87" t="s">
+      <c r="B2" s="97" t="s">
         <v>520</v>
       </c>
-      <c r="C2" s="87"/>
-      <c r="D2" s="87"/>
+      <c r="C2" s="97"/>
+      <c r="D2" s="97"/>
     </row>
     <row r="3" spans="2:7" ht="17.5" thickBot="1"/>
     <row r="4" spans="2:7" ht="21" customHeight="1" thickBot="1">
@@ -11059,16 +11295,16 @@
     <col min="2" max="2" width="27.33203125" customWidth="1"/>
     <col min="3" max="3" width="11.58203125" customWidth="1"/>
     <col min="4" max="4" width="61.08203125" customWidth="1"/>
-    <col min="5" max="5" width="83.1640625" customWidth="1"/>
+    <col min="5" max="5" width="83.08203125" customWidth="1"/>
     <col min="6" max="6" width="13.25" customWidth="1"/>
     <col min="7" max="7" width="41.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:7">
-      <c r="D1" s="88" t="s">
+      <c r="D1" s="98" t="s">
         <v>647</v>
       </c>
-      <c r="E1" s="88"/>
+      <c r="E1" s="98"/>
     </row>
     <row r="3" spans="2:7" ht="20.5">
       <c r="B3" s="60" t="s">
@@ -12365,8 +12601,8 @@
     <col min="2" max="2" width="8.25" style="26" customWidth="1"/>
     <col min="3" max="3" width="47.58203125" style="26" customWidth="1"/>
     <col min="4" max="5" width="13.83203125" style="26" customWidth="1"/>
-    <col min="7" max="7" width="8.6640625" customWidth="1"/>
-    <col min="8" max="8" width="15.6640625" customWidth="1"/>
+    <col min="7" max="7" width="8.58203125" customWidth="1"/>
+    <col min="8" max="8" width="15.58203125" customWidth="1"/>
     <col min="9" max="9" width="42.08203125" customWidth="1"/>
     <col min="10" max="10" width="47.58203125" customWidth="1"/>
   </cols>
@@ -13414,11 +13650,11 @@
   <dimension ref="B2:L53"/>
   <sheetFormatPr defaultRowHeight="17"/>
   <cols>
-    <col min="2" max="2" width="15.1640625" style="26" customWidth="1"/>
-    <col min="3" max="3" width="54.4140625" style="26" customWidth="1"/>
-    <col min="6" max="6" width="15.1640625" customWidth="1"/>
-    <col min="7" max="7" width="84.4140625" customWidth="1"/>
-    <col min="8" max="8" width="10.6640625" customWidth="1"/>
+    <col min="2" max="2" width="15.08203125" style="26" customWidth="1"/>
+    <col min="3" max="3" width="54.33203125" style="26" customWidth="1"/>
+    <col min="6" max="6" width="15.08203125" customWidth="1"/>
+    <col min="7" max="7" width="84.33203125" customWidth="1"/>
+    <col min="8" max="8" width="10.58203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:12" ht="20.5">
@@ -13636,7 +13872,7 @@
       <c r="C13" s="25" t="s">
         <v>818</v>
       </c>
-      <c r="E13" s="97"/>
+      <c r="E13" s="16"/>
       <c r="F13" s="25" t="s">
         <v>319</v>
       </c>
@@ -13738,7 +13974,7 @@
         <v>354</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>825</v>
+        <v>1080</v>
       </c>
       <c r="E18" s="16"/>
       <c r="F18" s="25" t="s">
@@ -13831,6 +14067,10 @@
       </c>
     </row>
     <row r="23" spans="2:12">
+      <c r="B23" s="100" t="s">
+        <v>1036</v>
+      </c>
+      <c r="C23" s="100"/>
       <c r="E23" s="16"/>
       <c r="F23" s="25" t="s">
         <v>154</v>
@@ -13846,6 +14086,10 @@
       </c>
     </row>
     <row r="24" spans="2:12">
+      <c r="B24" s="99" t="s">
+        <v>1091</v>
+      </c>
+      <c r="C24" s="99"/>
       <c r="E24" s="16"/>
       <c r="F24" s="25" t="s">
         <v>835</v>
@@ -13861,6 +14105,12 @@
       </c>
     </row>
     <row r="25" spans="2:12">
+      <c r="B25" s="25" t="s">
+        <v>1092</v>
+      </c>
+      <c r="C25" s="25" t="s">
+        <v>1093</v>
+      </c>
       <c r="E25" s="16"/>
       <c r="F25" s="25" t="s">
         <v>836</v>
@@ -13876,6 +14126,12 @@
       </c>
     </row>
     <row r="26" spans="2:12">
+      <c r="B26" s="25" t="s">
+        <v>1062</v>
+      </c>
+      <c r="C26" s="25" t="s">
+        <v>1103</v>
+      </c>
       <c r="E26" s="16" t="s">
         <v>1013</v>
       </c>
@@ -13893,6 +14149,10 @@
       </c>
     </row>
     <row r="27" spans="2:12">
+      <c r="B27" s="99" t="s">
+        <v>1094</v>
+      </c>
+      <c r="C27" s="99"/>
       <c r="E27" s="16"/>
       <c r="F27" s="25" t="s">
         <v>837</v>
@@ -13908,6 +14168,12 @@
       </c>
     </row>
     <row r="28" spans="2:12">
+      <c r="B28" s="25" t="s">
+        <v>1092</v>
+      </c>
+      <c r="C28" s="25" t="s">
+        <v>1095</v>
+      </c>
       <c r="E28" s="16"/>
       <c r="F28" s="25" t="s">
         <v>838</v>
@@ -13923,6 +14189,12 @@
       </c>
     </row>
     <row r="29" spans="2:12">
+      <c r="B29" s="25" t="s">
+        <v>1062</v>
+      </c>
+      <c r="C29" s="25" t="s">
+        <v>1096</v>
+      </c>
       <c r="E29" s="16"/>
       <c r="F29" s="25" t="s">
         <v>840</v>
@@ -13950,6 +14222,10 @@
       </c>
     </row>
     <row r="31" spans="2:12">
+      <c r="B31" s="100" t="s">
+        <v>1037</v>
+      </c>
+      <c r="C31" s="100"/>
       <c r="E31" s="16"/>
       <c r="F31" s="25" t="s">
         <v>1014</v>
@@ -13962,6 +14238,10 @@
       </c>
     </row>
     <row r="32" spans="2:12">
+      <c r="B32" s="99" t="s">
+        <v>1097</v>
+      </c>
+      <c r="C32" s="99"/>
       <c r="E32" s="16" t="s">
         <v>1013</v>
       </c>
@@ -13975,7 +14255,13 @@
         <v>2928</v>
       </c>
     </row>
-    <row r="33" spans="5:8">
+    <row r="33" spans="2:8">
+      <c r="B33" s="25" t="s">
+        <v>1100</v>
+      </c>
+      <c r="C33" s="25" t="s">
+        <v>1101</v>
+      </c>
       <c r="E33" s="16"/>
       <c r="F33" s="25" t="s">
         <v>844</v>
@@ -13987,7 +14273,11 @@
         <v>3288</v>
       </c>
     </row>
-    <row r="34" spans="5:8">
+    <row r="34" spans="2:8">
+      <c r="B34" s="25" t="s">
+        <v>1099</v>
+      </c>
+      <c r="C34" s="25"/>
       <c r="E34" s="16"/>
       <c r="F34" s="25" t="s">
         <v>119</v>
@@ -13999,7 +14289,11 @@
         <v>1615</v>
       </c>
     </row>
-    <row r="35" spans="5:8">
+    <row r="35" spans="2:8">
+      <c r="B35" s="99" t="s">
+        <v>1098</v>
+      </c>
+      <c r="C35" s="99"/>
       <c r="E35" s="16" t="s">
         <v>1013</v>
       </c>
@@ -14013,7 +14307,11 @@
         <v>2199</v>
       </c>
     </row>
-    <row r="36" spans="5:8">
+    <row r="36" spans="2:8">
+      <c r="B36" s="25" t="s">
+        <v>1100</v>
+      </c>
+      <c r="C36" s="25"/>
       <c r="E36" s="16"/>
       <c r="F36" s="25" t="s">
         <v>847</v>
@@ -14025,7 +14323,11 @@
         <v>5367</v>
       </c>
     </row>
-    <row r="37" spans="5:8">
+    <row r="37" spans="2:8">
+      <c r="B37" s="25" t="s">
+        <v>1099</v>
+      </c>
+      <c r="C37" s="25"/>
       <c r="E37" s="16"/>
       <c r="F37" s="25" t="s">
         <v>848</v>
@@ -14037,7 +14339,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="38" spans="5:8">
+    <row r="38" spans="2:8">
       <c r="E38" s="16" t="s">
         <v>1013</v>
       </c>
@@ -14051,7 +14353,13 @@
         <v>1444</v>
       </c>
     </row>
-    <row r="39" spans="5:8">
+    <row r="39" spans="2:8">
+      <c r="B39" s="101" t="s">
+        <v>1102</v>
+      </c>
+      <c r="C39" s="26" t="s">
+        <v>1082</v>
+      </c>
       <c r="E39" s="16"/>
       <c r="F39" s="25" t="s">
         <v>398</v>
@@ -14063,7 +14371,7 @@
         <v>3960</v>
       </c>
     </row>
-    <row r="40" spans="5:8">
+    <row r="40" spans="2:8">
       <c r="E40" s="16"/>
       <c r="F40" s="25" t="s">
         <v>433</v>
@@ -14075,7 +14383,7 @@
         <v>5030</v>
       </c>
     </row>
-    <row r="41" spans="5:8">
+    <row r="41" spans="2:8">
       <c r="E41" s="16" t="s">
         <v>1013</v>
       </c>
@@ -14089,7 +14397,7 @@
         <v>788</v>
       </c>
     </row>
-    <row r="42" spans="5:8">
+    <row r="42" spans="2:8">
       <c r="E42" s="16"/>
       <c r="F42" s="25" t="s">
         <v>325</v>
@@ -14101,7 +14409,7 @@
         <v>1190</v>
       </c>
     </row>
-    <row r="43" spans="5:8">
+    <row r="43" spans="2:8">
       <c r="E43" s="16" t="s">
         <v>1013</v>
       </c>
@@ -14115,7 +14423,7 @@
         <v>1443</v>
       </c>
     </row>
-    <row r="44" spans="5:8">
+    <row r="44" spans="2:8">
       <c r="E44" s="16" t="s">
         <v>1013</v>
       </c>
@@ -14129,7 +14437,7 @@
         <v>1588</v>
       </c>
     </row>
-    <row r="45" spans="5:8">
+    <row r="45" spans="2:8">
       <c r="E45" s="16" t="s">
         <v>1013</v>
       </c>
@@ -14143,7 +14451,7 @@
         <v>1441</v>
       </c>
     </row>
-    <row r="46" spans="5:8">
+    <row r="46" spans="2:8">
       <c r="E46" s="16"/>
       <c r="F46" s="25" t="s">
         <v>855</v>
@@ -14155,7 +14463,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="47" spans="5:8">
+    <row r="47" spans="2:8">
       <c r="E47" s="16"/>
       <c r="F47" s="25" t="s">
         <v>259</v>
@@ -14167,7 +14475,7 @@
         <v>4576</v>
       </c>
     </row>
-    <row r="48" spans="5:8">
+    <row r="48" spans="2:8">
       <c r="E48" s="16"/>
       <c r="F48" s="25" t="s">
         <v>856</v>
@@ -14242,6 +14550,14 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+  </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>